<commit_message>
Banking: fix a double semicolon in Chase; say Brex and the internal build offer no venture debt
Also make the deploy script's README check idempotent across chained edits.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build/startup-tool-stack-v3.xlsx
+++ b/build/startup-tool-stack-v3.xlsx
@@ -15774,7 +15774,7 @@
       </c>
       <c r="D236" s="14" t="inlineStr">
         <is>
-          <t>Cards are Visa or Mastercard cards issued by Emigrant Bank or Fifth Third Bank. Daily payments track your available balance; monthly payments run a 30-day statement and need $50,000 in cash if you have raised money. There is no personal guarantee, and limits are set on revenue and cash balance rather than a personal credit score. Points are 7x on rideshare, 4x on Brex-booked travel, 3x at restaurants, 2x on recurring software and 1x elsewhere, redeemed at 0.6 cents per point in cash. Unlimited virtual cards come on the $0 plan; expense policies need Premium at $12 per user.</t>
+          <t>Cards are Visa or Mastercard cards issued by Emigrant Bank or Fifth Third Bank. Daily payments track your available balance; monthly payments run a 30-day statement and need $50,000 in cash if you have raised money. There is no personal guarantee, and limits are set on revenue and cash balance rather than a personal credit score. Points are 7x on rideshare, 4x on Brex-booked travel, 3x at restaurants, 2x on recurring software and 1x elsewhere, redeemed at 0.6 cents per point in cash. Unlimited virtual cards come on the $0 plan; expense policies need Premium at $12 per user. No venture debt or line of credit is described.</t>
         </is>
       </c>
       <c r="E236" s="14" t="inlineStr">
@@ -15789,7 +15789,7 @@
       </c>
       <c r="G236" s="14" t="inlineStr">
         <is>
-          <t>Business Complete Checking comes with a debit card ($10,000 daily purchase limit) and employee debit access through the Business Associate Card at $0 annual fee. Credit is the Ink line (5 October 2026): Ink Business Unlimited has a $0 annual fee and 1.5% cash back;; Ink Business Premier costs $195 with 2% back and 2.5% on purchases of $5,000 or more. The Ink Business Unlimited terms make you and the business jointly responsible for the balance. A line of credit of $10,000 to $500,000 needs $100,000 in annual revenue, a FICO score of at least 660 and a personal guarantee from 20% owners.</t>
+          <t>Business Complete Checking comes with a debit card ($10,000 daily purchase limit) and employee debit access through the Business Associate Card at $0 annual fee. Credit is the Ink line (5 October 2026): Ink Business Unlimited has a $0 annual fee and 1.5% cash back; Ink Business Premier costs $195 with 2% back and 2.5% on purchases of $5,000 or more. The Ink Business Unlimited terms make you and the business jointly responsible for the balance. A line of credit of $10,000 to $500,000 needs $100,000 in annual revenue, a FICO score of at least 660 and a personal guarantee from 20% owners.</t>
         </is>
       </c>
       <c r="H236" s="14" t="inlineStr">
@@ -15799,7 +15799,7 @@
       </c>
       <c r="I236" s="14" t="inlineStr">
         <is>
-          <t>The deposit accounts come with a business debit card and employee debit cards and nothing else. There is no charge card, no cashback and no virtual cards; business credit cards and lines of credit are separate applications whose terms the sources used here do not state. Bank of America's employee debit cards default to a $400 daily purchase limit, adjustable to $7,500; Wells Fargo lets you adjust daily limits and turn a card on or off. That is the whole control surface: a daily cap and a switch, with no category blocks, merchant locks or receipt matching.</t>
+          <t>The deposit accounts come with a business debit card and employee debit cards and nothing else. There is no charge card, no cashback and no virtual cards; business credit cards and lines of credit are separate applications whose terms the sources used here do not state, and venture debt is not part of this route. Bank of America's employee debit cards default to a $400 daily purchase limit, adjustable to $7,500; Wells Fargo lets you adjust daily limits and turn a card on or off. That is the whole control surface: a daily cap and a switch, with no category blocks, merchant locks or receipt matching.</t>
         </is>
       </c>
       <c r="J236" s="10" t="n"/>

</xml_diff>